<commit_message>
Flag Gmail contacts as Validar 1º in weekly plan
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JJ31mnUiCbVaTaKMZZQpVz
</commit_message>
<xml_diff>
--- a/Plan_Correos_Semana_19-23Oct-2026.xlsx
+++ b/Plan_Correos_Semana_19-23Oct-2026.xlsx
@@ -565,7 +565,6 @@
           <t>En Calificación</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
         <v>1</v>
       </c>
@@ -619,7 +618,6 @@
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
         <v>3</v>
       </c>
@@ -731,7 +729,6 @@
           <t>En Calificación</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
         <v>3</v>
       </c>
@@ -785,7 +782,6 @@
           <t>En Calificación</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
         <v>1</v>
       </c>
@@ -955,7 +951,6 @@
           <t>En Calificación</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
         <v>1</v>
       </c>
@@ -1299,7 +1294,6 @@
           <t>En Calificación</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
         <v>2</v>
       </c>
@@ -1469,7 +1463,6 @@
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="n">
         <v>1</v>
       </c>
@@ -1523,7 +1516,6 @@
           <t>En Calificación</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
         <v>2</v>
       </c>
@@ -1577,7 +1569,6 @@
           <t>En Calificación</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
         <v>1</v>
       </c>
@@ -1873,7 +1864,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>En espera</t>
+          <t>Validar 1º</t>
         </is>
       </c>
     </row>
@@ -1931,7 +1922,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>En espera</t>
+          <t>Validar 1º</t>
         </is>
       </c>
     </row>

</xml_diff>